<commit_message>
Add CSR_Example, and update the format
</commit_message>
<xml_diff>
--- a/CSR_FORMAT_PROPOSAL.xlsx
+++ b/CSR_FORMAT_PROPOSAL.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27712"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\AppData\Roaming\MobaXterm\slash\RemoteFiles\66454_2_0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\002_GitHub\APB-CSR-Generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{152145C0-FF29-4FFC-9F71-23CE329CB6E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CE83735-1884-4388-9622-8E94304C9386}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DE80DA28-ED5E-4F9B-81E9-F3E91ABAB1A9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DE80DA28-ED5E-4F9B-81E9-F3E91ABAB1A9}"/>
   </bookViews>
   <sheets>
-    <sheet name="CSR_ASYNC" sheetId="6" r:id="rId1"/>
+    <sheet name="ASYNC_CSR" sheetId="6" r:id="rId1"/>
     <sheet name="CSR" sheetId="5" r:id="rId2"/>
     <sheet name="Register_Description" sheetId="7" r:id="rId3"/>
   </sheets>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="62">
   <si>
     <t>Table - Configuration</t>
   </si>
@@ -223,6 +223,9 @@
   </si>
   <si>
     <t>We are VLSI Technology</t>
+  </si>
+  <si>
+    <t>m_vlsi_async_csr</t>
   </si>
 </sst>
 </file>
@@ -326,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -336,8 +339,24 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -739,23 +758,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1BE8D60-EEB2-4162-9272-A435C8FC0492}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -766,18 +785,18 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -788,7 +807,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -799,7 +818,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -810,7 +829,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -821,7 +840,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -832,13 +851,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
@@ -861,7 +880,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -876,7 +895,7 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
@@ -893,7 +912,7 @@
       </c>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
@@ -910,7 +929,7 @@
       </c>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
@@ -927,7 +946,7 @@
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
@@ -944,7 +963,7 @@
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
@@ -961,7 +980,7 @@
       </c>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
@@ -978,7 +997,7 @@
       </c>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -993,7 +1012,7 @@
       </c>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
@@ -1010,7 +1029,7 @@
       </c>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
@@ -1027,7 +1046,7 @@
       </c>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
@@ -1044,7 +1063,7 @@
       </c>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
@@ -1061,7 +1080,7 @@
       </c>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
@@ -1078,7 +1097,7 @@
       </c>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
@@ -1103,23 +1122,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C536435B-4952-47A6-8C0D-14959CBB6C5F}">
   <dimension ref="A1:G29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>32</v>
       </c>
@@ -1130,7 +1149,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1141,7 +1160,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -1152,7 +1171,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1163,7 +1182,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
@@ -1174,7 +1193,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="29" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -1185,7 +1204,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="87" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>31</v>
       </c>
@@ -1196,13 +1215,13 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B14" s="3"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" s="6" t="s">
         <v>10</v>
       </c>
@@ -1225,7 +1244,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>43</v>
       </c>
@@ -1240,7 +1259,7 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1" t="s">
@@ -1257,7 +1276,7 @@
       </c>
       <c r="G17" s="1"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1" t="s">
@@ -1274,7 +1293,7 @@
       </c>
       <c r="G18" s="1"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
@@ -1291,7 +1310,7 @@
       </c>
       <c r="G19" s="1"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
@@ -1308,7 +1327,7 @@
       </c>
       <c r="G20" s="1"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1" t="s">
@@ -1325,7 +1344,7 @@
       </c>
       <c r="G21" s="1"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1" t="s">
@@ -1342,7 +1361,7 @@
       </c>
       <c r="G22" s="1"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
@@ -1357,7 +1376,7 @@
       </c>
       <c r="G23" s="1"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1" t="s">
@@ -1374,7 +1393,7 @@
       </c>
       <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1" t="s">
@@ -1391,7 +1410,7 @@
       </c>
       <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1" t="s">
@@ -1408,7 +1427,7 @@
       </c>
       <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1" t="s">
@@ -1425,7 +1444,7 @@
       </c>
       <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1" t="s">
@@ -1442,7 +1461,7 @@
       </c>
       <c r="G28" s="1"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1" t="s">
@@ -1468,103 +1487,106 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E03728AD-7351-4FF4-BFD8-5CD934512011}">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="44" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" style="8"/>
+    <col min="2" max="2" width="26.81640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" style="8"/>
+    <col min="4" max="4" width="44" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.7265625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="8"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="B1" s="7"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="B2" s="8"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="B2" s="7"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B3" s="8"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="B3" s="7"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B5" s="7"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="B5" s="9"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="11">
         <v>1</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>2</v>
-      </c>
-      <c r="B8" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="11">
+        <v>2</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
+    <row r="9" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A9" s="11">
         <v>3</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="12" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
+    <row r="10" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+      <c r="A10" s="11">
         <v>4</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="12" t="s">
         <v>55</v>
       </c>
     </row>

</xml_diff>